<commit_message>
docs(qms): approvals AR-2026-007 and AR-2026-008
Alexander Peter (review), Kishan Haravu Pradeep (data protection, AR-008),
Sheryl Nazareth (QA) and Anita Johan (Managing Director) confirmed on
2026-10-20:

- AR-2026-007: revision 1.1 of EM26-24 Test Plan, EM26-26 Use Cases,
  EM26-27 Client Communication Record and Log, EM26-30 Requirement Change
  Record, EM26-31 Design and Development Record; EM26-33 process,
  EM26-34 test execution register, release notes RN-v1.0.0 … v1.4.1
- AR-2026-008: EM26-35 AI Impact Assessment, SOP-05 rev 1.2 (§7a),
  REG-03 R-15 … R-18 and O-05, response to audit finding 6 (OFI-2026-06)

REG-01, QM-01, REG-03, REG-04 updated; audit pack documents signed;
QMS Word copies regenerated. OFI-2026-06 stays open until effectiveness
is verified at the internal audit.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/EchoMind_Audit_2026-10-14_Project2/03_Communication_with_Client/EM26-27_Client_Communication_Log.xlsx
+++ b/docs/EchoMind_Audit_2026-10-14_Project2/03_Communication_with_Client/EM26-27_Client_Communication_Log.xlsx
@@ -1578,7 +1578,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Rev 1.1 issued for approval; rev 1.0 approved 2026-10-13 (AR-2026-005)</t>
+          <t>APPROVED — rev 1.1 2026-10-20 (AR-2026-007); rev 1.0 approved 2026-10-13 (AR-2026-005)</t>
         </is>
       </c>
     </row>
@@ -1626,7 +1626,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Alexander Peter (EchoMind Project Lead) — rev 1.1 to confirm</t>
+          <t>Alexander Peter (EchoMind Project Lead) — 2026-10-20</t>
         </is>
       </c>
     </row>
@@ -1638,7 +1638,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Sheryl Nazareth (QA / MR) — rev 1.1 to confirm</t>
+          <t>Sheryl Nazareth (QA / MR) — 2026-10-20</t>
         </is>
       </c>
     </row>
@@ -1650,7 +1650,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Anita Johan (Managing Director) — rev 1.1 to confirm</t>
+          <t>Anita Johan (Managing Director) — 2026-10-20</t>
         </is>
       </c>
     </row>

</xml_diff>